<commit_message>
feat: images added to excel generation
</commit_message>
<xml_diff>
--- a/SupervisorMobility.API/DataAccess/Templates/Analysis Template.xlsx
+++ b/SupervisorMobility.API/DataAccess/Templates/Analysis Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ituriel\OneDrive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A48DC56-BC47-4566-8690-29CBD705A89B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7F5C517-ECE2-4E36-9AF0-BD8DF00C3CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29280" yWindow="4125" windowWidth="25650" windowHeight="15285" xr2:uid="{D0212AFC-6A0E-4C55-A58F-05F4C514B5A6}"/>
+    <workbookView xWindow="29745" yWindow="3840" windowWidth="25650" windowHeight="15285" xr2:uid="{D0212AFC-6A0E-4C55-A58F-05F4C514B5A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Analysis A" sheetId="1" r:id="rId1"/>
@@ -1028,7 +1028,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="126">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1106,23 +1106,68 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1130,14 +1175,71 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1230,150 +1332,83 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1729,163 +1764,163 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:17" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="52" t="s">
+      <c r="B3" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="52"/>
-      <c r="J3" s="52"/>
+      <c r="C3" s="86"/>
+      <c r="D3" s="86"/>
+      <c r="E3" s="86"/>
+      <c r="F3" s="86"/>
+      <c r="G3" s="86"/>
+      <c r="H3" s="86"/>
+      <c r="I3" s="86"/>
+      <c r="J3" s="86"/>
     </row>
     <row r="4" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="53" t="s">
+      <c r="B4" s="87" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="59"/>
-      <c r="H4" s="63" t="s">
+      <c r="C4" s="88"/>
+      <c r="D4" s="91"/>
+      <c r="E4" s="92"/>
+      <c r="F4" s="92"/>
+      <c r="G4" s="93"/>
+      <c r="H4" s="97" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="64"/>
-      <c r="J4" s="56"/>
-      <c r="K4" s="80"/>
-      <c r="L4" s="81"/>
-      <c r="M4" s="82"/>
+      <c r="I4" s="98"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="61"/>
+      <c r="L4" s="62"/>
+      <c r="M4" s="63"/>
       <c r="N4" s="12"/>
       <c r="O4" s="12"/>
       <c r="P4" s="11"/>
       <c r="Q4" s="14"/>
     </row>
     <row r="5" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="55"/>
-      <c r="C5" s="56"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="61"/>
-      <c r="F5" s="61"/>
-      <c r="G5" s="62"/>
-      <c r="H5" s="77" t="s">
+      <c r="B5" s="89"/>
+      <c r="C5" s="90"/>
+      <c r="D5" s="94"/>
+      <c r="E5" s="95"/>
+      <c r="F5" s="95"/>
+      <c r="G5" s="96"/>
+      <c r="H5" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="78"/>
-      <c r="J5" s="79"/>
-      <c r="K5" s="83"/>
-      <c r="L5" s="84"/>
-      <c r="M5" s="85"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="60"/>
+      <c r="K5" s="64"/>
+      <c r="L5" s="65"/>
+      <c r="M5" s="66"/>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
       <c r="P5" s="5"/>
       <c r="Q5" s="14"/>
     </row>
     <row r="6" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="86" t="s">
+      <c r="B6" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="79"/>
-      <c r="D6" s="87"/>
-      <c r="E6" s="88"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="40"/>
       <c r="F6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="G6" s="3"/>
-      <c r="H6" s="93" t="s">
+      <c r="H6" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="94"/>
-      <c r="J6" s="109"/>
-      <c r="K6" s="116"/>
-      <c r="L6" s="116"/>
-      <c r="M6" s="116"/>
-      <c r="N6" s="117"/>
-      <c r="O6" s="118"/>
-      <c r="P6" s="90"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="50"/>
+      <c r="L6" s="50"/>
+      <c r="M6" s="50"/>
+      <c r="N6" s="52"/>
+      <c r="O6" s="53"/>
+      <c r="P6" s="68"/>
     </row>
     <row r="7" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="86" t="s">
+      <c r="B7" s="67" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="79"/>
-      <c r="D7" s="87"/>
-      <c r="E7" s="89"/>
-      <c r="F7" s="89"/>
-      <c r="G7" s="88"/>
-      <c r="H7" s="110"/>
-      <c r="I7" s="111"/>
-      <c r="J7" s="112"/>
-      <c r="K7" s="116"/>
-      <c r="L7" s="116"/>
-      <c r="M7" s="116"/>
-      <c r="N7" s="117"/>
-      <c r="O7" s="119"/>
-      <c r="P7" s="91"/>
+      <c r="C7" s="60"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="40"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="45"/>
+      <c r="J7" s="46"/>
+      <c r="K7" s="50"/>
+      <c r="L7" s="50"/>
+      <c r="M7" s="50"/>
+      <c r="N7" s="52"/>
+      <c r="O7" s="54"/>
+      <c r="P7" s="69"/>
     </row>
     <row r="8" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="86" t="s">
+      <c r="B8" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="79"/>
-      <c r="D8" s="87"/>
-      <c r="E8" s="89"/>
-      <c r="F8" s="89"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="113"/>
-      <c r="I8" s="114"/>
-      <c r="J8" s="115"/>
-      <c r="K8" s="105"/>
-      <c r="L8" s="105"/>
-      <c r="M8" s="105"/>
-      <c r="N8" s="117"/>
-      <c r="O8" s="120"/>
-      <c r="P8" s="92"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="47"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="49"/>
+      <c r="K8" s="51"/>
+      <c r="L8" s="51"/>
+      <c r="M8" s="51"/>
+      <c r="N8" s="52"/>
+      <c r="O8" s="55"/>
+      <c r="P8" s="70"/>
     </row>
     <row r="9" spans="1:17" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10"/>
-      <c r="B9" s="78" t="s">
+      <c r="B9" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="79"/>
-      <c r="D9" s="87"/>
-      <c r="E9" s="89"/>
-      <c r="F9" s="89"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="97" t="s">
+      <c r="C9" s="60"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="40"/>
+      <c r="H9" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="93" t="s">
+      <c r="I9" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="J9" s="94"/>
-      <c r="K9" s="104"/>
-      <c r="L9" s="105"/>
-      <c r="M9" s="105"/>
+      <c r="J9" s="42"/>
+      <c r="K9" s="111"/>
+      <c r="L9" s="51"/>
+      <c r="M9" s="51"/>
       <c r="N9" s="6"/>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="14"/>
     </row>
     <row r="10" spans="1:17" ht="46.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="99" t="s">
+      <c r="B10" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="100"/>
-      <c r="D10" s="101"/>
-      <c r="E10" s="102"/>
-      <c r="F10" s="102"/>
-      <c r="G10" s="103"/>
-      <c r="H10" s="98"/>
-      <c r="I10" s="95" t="s">
+      <c r="C10" s="76"/>
+      <c r="D10" s="77"/>
+      <c r="E10" s="78"/>
+      <c r="F10" s="78"/>
+      <c r="G10" s="79"/>
+      <c r="H10" s="74"/>
+      <c r="I10" s="71" t="s">
         <v>10</v>
       </c>
-      <c r="J10" s="96"/>
-      <c r="K10" s="106"/>
-      <c r="L10" s="107"/>
-      <c r="M10" s="108"/>
+      <c r="J10" s="72"/>
+      <c r="K10" s="112"/>
+      <c r="L10" s="113"/>
+      <c r="M10" s="114"/>
       <c r="N10" s="13"/>
       <c r="O10" s="8"/>
       <c r="P10" s="13"/>
@@ -1901,53 +1936,53 @@
       <c r="P11" s="9"/>
     </row>
     <row r="12" spans="1:17" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="65" t="s">
+      <c r="B12" s="99" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="67" t="s">
+      <c r="C12" s="101" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="68"/>
-      <c r="E12" s="71" t="s">
+      <c r="D12" s="102"/>
+      <c r="E12" s="105" t="s">
         <v>14</v>
       </c>
-      <c r="F12" s="67" t="s">
+      <c r="F12" s="101" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="68"/>
-      <c r="H12" s="73" t="s">
+      <c r="G12" s="102"/>
+      <c r="H12" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="73"/>
-      <c r="J12" s="67" t="s">
+      <c r="I12" s="107"/>
+      <c r="J12" s="101" t="s">
         <v>20</v>
       </c>
-      <c r="K12" s="73"/>
-      <c r="L12" s="74"/>
-      <c r="M12" s="41" t="s">
+      <c r="K12" s="107"/>
+      <c r="L12" s="108"/>
+      <c r="M12" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="N12" s="42"/>
-      <c r="O12" s="42"/>
-      <c r="P12" s="42"/>
+      <c r="N12" s="57"/>
+      <c r="O12" s="57"/>
+      <c r="P12" s="57"/>
       <c r="Q12" s="14"/>
     </row>
     <row r="13" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="66"/>
-      <c r="C13" s="69"/>
-      <c r="D13" s="70"/>
-      <c r="E13" s="72"/>
-      <c r="F13" s="69"/>
-      <c r="G13" s="70"/>
+      <c r="B13" s="100"/>
+      <c r="C13" s="103"/>
+      <c r="D13" s="104"/>
+      <c r="E13" s="106"/>
+      <c r="F13" s="103"/>
+      <c r="G13" s="104"/>
       <c r="H13" s="17" t="s">
         <v>18</v>
       </c>
       <c r="I13" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="69"/>
-      <c r="K13" s="75"/>
-      <c r="L13" s="76"/>
+      <c r="J13" s="103"/>
+      <c r="K13" s="109"/>
+      <c r="L13" s="110"/>
       <c r="M13" s="16"/>
       <c r="N13" s="9"/>
       <c r="O13" s="9"/>
@@ -1955,29 +1990,29 @@
     </row>
     <row r="14" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="34"/>
-      <c r="C14" s="46"/>
-      <c r="D14" s="49"/>
+      <c r="C14" s="125"/>
+      <c r="D14" s="131"/>
       <c r="E14" s="20"/>
-      <c r="F14" s="50"/>
-      <c r="G14" s="51"/>
+      <c r="F14" s="133"/>
+      <c r="G14" s="134"/>
       <c r="H14" s="18"/>
       <c r="I14" s="19"/>
-      <c r="J14" s="46"/>
-      <c r="K14" s="47"/>
-      <c r="L14" s="48"/>
+      <c r="J14" s="125"/>
+      <c r="K14" s="126"/>
+      <c r="L14" s="127"/>
     </row>
     <row r="15" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="21"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
+      <c r="C15" s="128"/>
+      <c r="D15" s="132"/>
       <c r="E15" s="22"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="38"/>
+      <c r="F15" s="135"/>
+      <c r="G15" s="136"/>
       <c r="H15" s="23"/>
       <c r="I15" s="24"/>
-      <c r="J15" s="35"/>
-      <c r="K15" s="39"/>
-      <c r="L15" s="40"/>
+      <c r="J15" s="128"/>
+      <c r="K15" s="129"/>
+      <c r="L15" s="130"/>
     </row>
     <row r="16" spans="1:17" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="27"/>
@@ -1999,35 +2034,53 @@
       <c r="L17" s="26"/>
     </row>
     <row r="18" spans="2:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="41" t="s">
+      <c r="B18" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="42"/>
-      <c r="D18" s="42"/>
+      <c r="C18" s="57"/>
+      <c r="D18" s="57"/>
       <c r="E18" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="F18" s="43" t="s">
+      <c r="F18" s="122" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="42"/>
-      <c r="H18" s="43" t="s">
+      <c r="G18" s="57"/>
+      <c r="H18" s="122" t="s">
         <v>26</v>
       </c>
-      <c r="I18" s="42"/>
-      <c r="J18" s="44"/>
-      <c r="K18" s="42" t="s">
+      <c r="I18" s="57"/>
+      <c r="J18" s="123"/>
+      <c r="K18" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="L18" s="45"/>
+      <c r="L18" s="121"/>
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="H6:J8"/>
-    <mergeCell ref="K6:M8"/>
-    <mergeCell ref="N6:N8"/>
-    <mergeCell ref="O6:O8"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="J15:L15"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="D4:G5"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="F12:G13"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="J12:L13"/>
+    <mergeCell ref="K9:M9"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="B8:C8"/>
     <mergeCell ref="M12:P12"/>
     <mergeCell ref="H5:J5"/>
     <mergeCell ref="K4:M4"/>
@@ -2044,29 +2097,11 @@
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="D10:G10"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="B4:C5"/>
-    <mergeCell ref="D4:G5"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="F12:G13"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J12:L13"/>
-    <mergeCell ref="K9:M9"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="H6:J8"/>
+    <mergeCell ref="K6:M8"/>
+    <mergeCell ref="N6:N8"/>
+    <mergeCell ref="O6:O8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2106,88 +2141,81 @@
       <c r="I3" s="124"/>
       <c r="J3" s="124"/>
     </row>
-    <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="N4" s="122"/>
-      <c r="O4" s="122"/>
-      <c r="P4" s="122"/>
-    </row>
+    <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="65" t="s">
+      <c r="B5" s="99" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="67" t="s">
+      <c r="C5" s="101" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="68"/>
-      <c r="E5" s="71" t="s">
+      <c r="D5" s="102"/>
+      <c r="E5" s="105" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="67" t="s">
+      <c r="F5" s="101" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="68"/>
-      <c r="H5" s="73" t="s">
+      <c r="G5" s="102"/>
+      <c r="H5" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="73"/>
-      <c r="J5" s="67" t="s">
+      <c r="I5" s="107"/>
+      <c r="J5" s="101" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="73"/>
-      <c r="L5" s="74"/>
-      <c r="M5" s="121" t="s">
+      <c r="K5" s="107"/>
+      <c r="L5" s="108"/>
+      <c r="M5" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="N5" s="123"/>
-      <c r="O5" s="123"/>
-      <c r="P5" s="123"/>
+      <c r="N5" s="35"/>
+      <c r="O5" s="35"/>
+      <c r="P5" s="35"/>
     </row>
     <row r="6" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="66"/>
-      <c r="C6" s="69"/>
-      <c r="D6" s="70"/>
-      <c r="E6" s="72"/>
-      <c r="F6" s="69"/>
-      <c r="G6" s="70"/>
+      <c r="B6" s="100"/>
+      <c r="C6" s="103"/>
+      <c r="D6" s="104"/>
+      <c r="E6" s="106"/>
+      <c r="F6" s="103"/>
+      <c r="G6" s="104"/>
       <c r="H6" s="17" t="s">
         <v>18</v>
       </c>
       <c r="I6" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="69"/>
-      <c r="K6" s="75"/>
-      <c r="L6" s="76"/>
+      <c r="J6" s="103"/>
+      <c r="K6" s="109"/>
+      <c r="L6" s="110"/>
       <c r="M6" s="16"/>
-      <c r="N6" s="122"/>
-      <c r="O6" s="122"/>
-      <c r="P6" s="122"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B7" s="34"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="49"/>
+      <c r="C7" s="80"/>
+      <c r="D7" s="83"/>
       <c r="E7" s="20"/>
-      <c r="F7" s="50"/>
-      <c r="G7" s="51"/>
+      <c r="F7" s="84"/>
+      <c r="G7" s="85"/>
       <c r="H7" s="18"/>
       <c r="I7" s="19"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="47"/>
-      <c r="L7" s="48"/>
+      <c r="J7" s="80"/>
+      <c r="K7" s="81"/>
+      <c r="L7" s="82"/>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B8" s="21"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="36"/>
+      <c r="C8" s="115"/>
+      <c r="D8" s="116"/>
       <c r="E8" s="22"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="38"/>
+      <c r="F8" s="117"/>
+      <c r="G8" s="118"/>
       <c r="H8" s="23"/>
       <c r="I8" s="24"/>
-      <c r="J8" s="35"/>
-      <c r="K8" s="39"/>
-      <c r="L8" s="40"/>
+      <c r="J8" s="115"/>
+      <c r="K8" s="119"/>
+      <c r="L8" s="120"/>
     </row>
     <row r="9" spans="2:16" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="27"/>
@@ -2209,30 +2237,31 @@
       <c r="L10" s="26"/>
     </row>
     <row r="11" spans="2:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
+      <c r="C11" s="57"/>
+      <c r="D11" s="57"/>
       <c r="E11" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="43" t="s">
+      <c r="F11" s="122" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="42"/>
-      <c r="H11" s="43" t="s">
+      <c r="G11" s="57"/>
+      <c r="H11" s="122" t="s">
         <v>26</v>
       </c>
-      <c r="I11" s="42"/>
-      <c r="J11" s="44"/>
-      <c r="K11" s="42" t="s">
+      <c r="I11" s="57"/>
+      <c r="J11" s="123"/>
+      <c r="K11" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="L11" s="45"/>
+      <c r="L11" s="121"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="J5:L6"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="K11:L11"/>
     <mergeCell ref="B3:J3"/>
@@ -2249,7 +2278,6 @@
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="F5:G6"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:L6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2267,19 +2295,19 @@
   <sheetData>
     <row r="1" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="125" t="s">
+      <c r="A2" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="125" t="s">
+      <c r="C2" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="125" t="s">
+      <c r="D2" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="125" t="s">
+      <c r="E2" s="37" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: images now containes within max row height
</commit_message>
<xml_diff>
--- a/SupervisorMobility.API/DataAccess/Templates/Analysis Template.xlsx
+++ b/SupervisorMobility.API/DataAccess/Templates/Analysis Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ituriel\OneDrive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7F5C517-ECE2-4E36-9AF0-BD8DF00C3CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0390C311-95FE-4DA4-885B-F53CDC37E205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29745" yWindow="3840" windowWidth="25650" windowHeight="15285" xr2:uid="{D0212AFC-6A0E-4C55-A58F-05F4C514B5A6}"/>
+    <workbookView xWindow="29850" yWindow="2025" windowWidth="29835" windowHeight="16605" activeTab="1" xr2:uid="{D0212AFC-6A0E-4C55-A58F-05F4C514B5A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Analysis A" sheetId="1" r:id="rId1"/>
@@ -1115,14 +1115,192 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1130,90 +1308,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1241,109 +1335,63 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1361,54 +1409,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1764,163 +1764,163 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:17" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="55" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="86"/>
-      <c r="D3" s="86"/>
-      <c r="E3" s="86"/>
-      <c r="F3" s="86"/>
-      <c r="G3" s="86"/>
-      <c r="H3" s="86"/>
-      <c r="I3" s="86"/>
-      <c r="J3" s="86"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
     </row>
     <row r="4" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="87" t="s">
+      <c r="B4" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="88"/>
-      <c r="D4" s="91"/>
-      <c r="E4" s="92"/>
-      <c r="F4" s="92"/>
-      <c r="G4" s="93"/>
-      <c r="H4" s="97" t="s">
+      <c r="C4" s="57"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="98"/>
-      <c r="J4" s="90"/>
-      <c r="K4" s="61"/>
-      <c r="L4" s="62"/>
-      <c r="M4" s="63"/>
+      <c r="I4" s="67"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="89"/>
+      <c r="L4" s="90"/>
+      <c r="M4" s="91"/>
       <c r="N4" s="12"/>
       <c r="O4" s="12"/>
       <c r="P4" s="11"/>
       <c r="Q4" s="14"/>
     </row>
     <row r="5" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="89"/>
-      <c r="C5" s="90"/>
-      <c r="D5" s="94"/>
-      <c r="E5" s="95"/>
-      <c r="F5" s="95"/>
-      <c r="G5" s="96"/>
-      <c r="H5" s="58" t="s">
+      <c r="B5" s="58"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="63"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="65"/>
+      <c r="H5" s="87" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="59"/>
-      <c r="J5" s="60"/>
-      <c r="K5" s="64"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="66"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="86"/>
+      <c r="K5" s="92"/>
+      <c r="L5" s="93"/>
+      <c r="M5" s="94"/>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
       <c r="P5" s="5"/>
       <c r="Q5" s="14"/>
     </row>
     <row r="6" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="67" t="s">
+      <c r="B6" s="85" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="60"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="40"/>
+      <c r="C6" s="86"/>
+      <c r="D6" s="95"/>
+      <c r="E6" s="96"/>
       <c r="F6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="G6" s="3"/>
-      <c r="H6" s="41" t="s">
+      <c r="H6" s="101" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="42"/>
-      <c r="J6" s="43"/>
-      <c r="K6" s="50"/>
-      <c r="L6" s="50"/>
-      <c r="M6" s="50"/>
-      <c r="N6" s="52"/>
-      <c r="O6" s="53"/>
-      <c r="P6" s="68"/>
+      <c r="I6" s="102"/>
+      <c r="J6" s="112"/>
+      <c r="K6" s="119"/>
+      <c r="L6" s="119"/>
+      <c r="M6" s="119"/>
+      <c r="N6" s="120"/>
+      <c r="O6" s="121"/>
+      <c r="P6" s="98"/>
     </row>
     <row r="7" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="67" t="s">
+      <c r="B7" s="85" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="60"/>
-      <c r="D7" s="38"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
-      <c r="G7" s="40"/>
-      <c r="H7" s="44"/>
-      <c r="I7" s="45"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="50"/>
-      <c r="L7" s="50"/>
-      <c r="M7" s="50"/>
-      <c r="N7" s="52"/>
-      <c r="O7" s="54"/>
-      <c r="P7" s="69"/>
+      <c r="C7" s="86"/>
+      <c r="D7" s="95"/>
+      <c r="E7" s="97"/>
+      <c r="F7" s="97"/>
+      <c r="G7" s="96"/>
+      <c r="H7" s="113"/>
+      <c r="I7" s="114"/>
+      <c r="J7" s="115"/>
+      <c r="K7" s="119"/>
+      <c r="L7" s="119"/>
+      <c r="M7" s="119"/>
+      <c r="N7" s="120"/>
+      <c r="O7" s="122"/>
+      <c r="P7" s="99"/>
     </row>
     <row r="8" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="67" t="s">
+      <c r="B8" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="60"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="47"/>
-      <c r="I8" s="48"/>
-      <c r="J8" s="49"/>
-      <c r="K8" s="51"/>
-      <c r="L8" s="51"/>
-      <c r="M8" s="51"/>
-      <c r="N8" s="52"/>
-      <c r="O8" s="55"/>
-      <c r="P8" s="70"/>
+      <c r="C8" s="86"/>
+      <c r="D8" s="95"/>
+      <c r="E8" s="97"/>
+      <c r="F8" s="97"/>
+      <c r="G8" s="96"/>
+      <c r="H8" s="116"/>
+      <c r="I8" s="117"/>
+      <c r="J8" s="118"/>
+      <c r="K8" s="81"/>
+      <c r="L8" s="81"/>
+      <c r="M8" s="81"/>
+      <c r="N8" s="120"/>
+      <c r="O8" s="123"/>
+      <c r="P8" s="100"/>
     </row>
     <row r="9" spans="1:17" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10"/>
-      <c r="B9" s="59" t="s">
+      <c r="B9" s="88" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="60"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="40"/>
-      <c r="H9" s="73" t="s">
+      <c r="C9" s="86"/>
+      <c r="D9" s="95"/>
+      <c r="E9" s="97"/>
+      <c r="F9" s="97"/>
+      <c r="G9" s="96"/>
+      <c r="H9" s="105" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="41" t="s">
+      <c r="I9" s="101" t="s">
         <v>8</v>
       </c>
-      <c r="J9" s="42"/>
-      <c r="K9" s="111"/>
-      <c r="L9" s="51"/>
-      <c r="M9" s="51"/>
+      <c r="J9" s="102"/>
+      <c r="K9" s="80"/>
+      <c r="L9" s="81"/>
+      <c r="M9" s="81"/>
       <c r="N9" s="6"/>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="14"/>
     </row>
     <row r="10" spans="1:17" ht="46.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="75" t="s">
+      <c r="B10" s="107" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="76"/>
-      <c r="D10" s="77"/>
-      <c r="E10" s="78"/>
-      <c r="F10" s="78"/>
-      <c r="G10" s="79"/>
-      <c r="H10" s="74"/>
-      <c r="I10" s="71" t="s">
+      <c r="C10" s="108"/>
+      <c r="D10" s="109"/>
+      <c r="E10" s="110"/>
+      <c r="F10" s="110"/>
+      <c r="G10" s="111"/>
+      <c r="H10" s="106"/>
+      <c r="I10" s="103" t="s">
         <v>10</v>
       </c>
-      <c r="J10" s="72"/>
-      <c r="K10" s="112"/>
-      <c r="L10" s="113"/>
-      <c r="M10" s="114"/>
+      <c r="J10" s="104"/>
+      <c r="K10" s="82"/>
+      <c r="L10" s="83"/>
+      <c r="M10" s="84"/>
       <c r="N10" s="13"/>
       <c r="O10" s="8"/>
       <c r="P10" s="13"/>
@@ -1936,53 +1936,53 @@
       <c r="P11" s="9"/>
     </row>
     <row r="12" spans="1:17" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="99" t="s">
+      <c r="B12" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="101" t="s">
+      <c r="C12" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="102"/>
-      <c r="E12" s="105" t="s">
+      <c r="D12" s="71"/>
+      <c r="E12" s="74" t="s">
         <v>14</v>
       </c>
-      <c r="F12" s="101" t="s">
+      <c r="F12" s="70" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="102"/>
-      <c r="H12" s="107" t="s">
+      <c r="G12" s="71"/>
+      <c r="H12" s="76" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="107"/>
-      <c r="J12" s="101" t="s">
+      <c r="I12" s="76"/>
+      <c r="J12" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="K12" s="107"/>
-      <c r="L12" s="108"/>
-      <c r="M12" s="56" t="s">
+      <c r="K12" s="76"/>
+      <c r="L12" s="77"/>
+      <c r="M12" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="N12" s="57"/>
-      <c r="O12" s="57"/>
-      <c r="P12" s="57"/>
+      <c r="N12" s="45"/>
+      <c r="O12" s="45"/>
+      <c r="P12" s="45"/>
       <c r="Q12" s="14"/>
     </row>
     <row r="13" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="100"/>
-      <c r="C13" s="103"/>
-      <c r="D13" s="104"/>
-      <c r="E13" s="106"/>
-      <c r="F13" s="103"/>
-      <c r="G13" s="104"/>
+      <c r="B13" s="69"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="73"/>
+      <c r="E13" s="75"/>
+      <c r="F13" s="72"/>
+      <c r="G13" s="73"/>
       <c r="H13" s="17" t="s">
         <v>18</v>
       </c>
       <c r="I13" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="103"/>
-      <c r="K13" s="109"/>
-      <c r="L13" s="110"/>
+      <c r="J13" s="72"/>
+      <c r="K13" s="78"/>
+      <c r="L13" s="79"/>
       <c r="M13" s="16"/>
       <c r="N13" s="9"/>
       <c r="O13" s="9"/>
@@ -1990,29 +1990,29 @@
     </row>
     <row r="14" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="34"/>
-      <c r="C14" s="125"/>
-      <c r="D14" s="131"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="52"/>
       <c r="E14" s="20"/>
-      <c r="F14" s="133"/>
-      <c r="G14" s="134"/>
+      <c r="F14" s="53"/>
+      <c r="G14" s="54"/>
       <c r="H14" s="18"/>
       <c r="I14" s="19"/>
-      <c r="J14" s="125"/>
-      <c r="K14" s="126"/>
-      <c r="L14" s="127"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="50"/>
+      <c r="L14" s="51"/>
     </row>
     <row r="15" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="21"/>
-      <c r="C15" s="128"/>
-      <c r="D15" s="132"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="39"/>
       <c r="E15" s="22"/>
-      <c r="F15" s="135"/>
-      <c r="G15" s="136"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="41"/>
       <c r="H15" s="23"/>
       <c r="I15" s="24"/>
-      <c r="J15" s="128"/>
-      <c r="K15" s="129"/>
-      <c r="L15" s="130"/>
+      <c r="J15" s="38"/>
+      <c r="K15" s="42"/>
+      <c r="L15" s="43"/>
     </row>
     <row r="16" spans="1:17" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="27"/>
@@ -2034,37 +2034,51 @@
       <c r="L17" s="26"/>
     </row>
     <row r="18" spans="2:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="56" t="s">
+      <c r="B18" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="57"/>
-      <c r="D18" s="57"/>
+      <c r="C18" s="45"/>
+      <c r="D18" s="45"/>
       <c r="E18" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="F18" s="122" t="s">
+      <c r="F18" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="57"/>
-      <c r="H18" s="122" t="s">
+      <c r="G18" s="45"/>
+      <c r="H18" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="I18" s="57"/>
-      <c r="J18" s="123"/>
-      <c r="K18" s="57" t="s">
+      <c r="I18" s="45"/>
+      <c r="J18" s="48"/>
+      <c r="K18" s="45" t="s">
         <v>27</v>
       </c>
-      <c r="L18" s="121"/>
+      <c r="L18" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="H6:J8"/>
+    <mergeCell ref="K6:M8"/>
+    <mergeCell ref="N6:N8"/>
+    <mergeCell ref="O6:O8"/>
+    <mergeCell ref="M12:P12"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="P6:P8"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="D10:G10"/>
     <mergeCell ref="J14:L14"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="F14:G14"/>
@@ -2081,27 +2095,13 @@
     <mergeCell ref="K9:M9"/>
     <mergeCell ref="K10:M10"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="M12:P12"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:G7"/>
-    <mergeCell ref="P6:P8"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D9:G9"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="H6:J8"/>
-    <mergeCell ref="K6:M8"/>
-    <mergeCell ref="N6:N8"/>
-    <mergeCell ref="O6:O8"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="J15:L15"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:J18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2143,29 +2143,29 @@
     </row>
     <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="99" t="s">
+      <c r="B5" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="101" t="s">
+      <c r="C5" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="102"/>
-      <c r="E5" s="105" t="s">
+      <c r="D5" s="71"/>
+      <c r="E5" s="74" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="101" t="s">
+      <c r="F5" s="70" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="102"/>
-      <c r="H5" s="107" t="s">
+      <c r="G5" s="71"/>
+      <c r="H5" s="76" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="107"/>
-      <c r="J5" s="101" t="s">
+      <c r="I5" s="76"/>
+      <c r="J5" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="107"/>
-      <c r="L5" s="108"/>
+      <c r="K5" s="76"/>
+      <c r="L5" s="77"/>
       <c r="M5" s="36" t="s">
         <v>21</v>
       </c>
@@ -2174,50 +2174,50 @@
       <c r="P5" s="35"/>
     </row>
     <row r="6" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="100"/>
-      <c r="C6" s="103"/>
-      <c r="D6" s="104"/>
-      <c r="E6" s="106"/>
-      <c r="F6" s="103"/>
-      <c r="G6" s="104"/>
+      <c r="B6" s="69"/>
+      <c r="C6" s="72"/>
+      <c r="D6" s="73"/>
+      <c r="E6" s="75"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="73"/>
       <c r="H6" s="17" t="s">
         <v>18</v>
       </c>
       <c r="I6" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="103"/>
-      <c r="K6" s="109"/>
-      <c r="L6" s="110"/>
+      <c r="J6" s="72"/>
+      <c r="K6" s="78"/>
+      <c r="L6" s="79"/>
       <c r="M6" s="16"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B7" s="34"/>
-      <c r="C7" s="80"/>
-      <c r="D7" s="83"/>
+      <c r="C7" s="125"/>
+      <c r="D7" s="126"/>
       <c r="E7" s="20"/>
-      <c r="F7" s="84"/>
-      <c r="G7" s="85"/>
+      <c r="F7" s="127"/>
+      <c r="G7" s="128"/>
       <c r="H7" s="18"/>
       <c r="I7" s="19"/>
-      <c r="J7" s="80"/>
-      <c r="K7" s="81"/>
-      <c r="L7" s="82"/>
+      <c r="J7" s="125"/>
+      <c r="K7" s="129"/>
+      <c r="L7" s="130"/>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B8" s="21"/>
-      <c r="C8" s="115"/>
-      <c r="D8" s="116"/>
+      <c r="C8" s="131"/>
+      <c r="D8" s="132"/>
       <c r="E8" s="22"/>
-      <c r="F8" s="117"/>
-      <c r="G8" s="118"/>
+      <c r="F8" s="133"/>
+      <c r="G8" s="134"/>
       <c r="H8" s="23"/>
       <c r="I8" s="24"/>
-      <c r="J8" s="115"/>
-      <c r="K8" s="119"/>
-      <c r="L8" s="120"/>
-    </row>
-    <row r="9" spans="2:16" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="J8" s="131"/>
+      <c r="K8" s="135"/>
+      <c r="L8" s="136"/>
+    </row>
+    <row r="9" spans="2:16" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="27"/>
       <c r="C9" s="28"/>
       <c r="D9" s="28"/>
@@ -2237,30 +2237,31 @@
       <c r="L10" s="26"/>
     </row>
     <row r="11" spans="2:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="56" t="s">
+      <c r="B11" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="57"/>
-      <c r="D11" s="57"/>
+      <c r="C11" s="45"/>
+      <c r="D11" s="45"/>
       <c r="E11" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="122" t="s">
+      <c r="F11" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="57"/>
-      <c r="H11" s="122" t="s">
+      <c r="G11" s="45"/>
+      <c r="H11" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="I11" s="57"/>
-      <c r="J11" s="123"/>
-      <c r="K11" s="57" t="s">
+      <c r="I11" s="45"/>
+      <c r="J11" s="48"/>
+      <c r="K11" s="45" t="s">
         <v>27</v>
       </c>
-      <c r="L11" s="121"/>
+      <c r="L11" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="H5:I5"/>
     <mergeCell ref="J5:L6"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="K11:L11"/>
@@ -2277,7 +2278,6 @@
     <mergeCell ref="C5:D6"/>
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="F5:G6"/>
-    <mergeCell ref="H5:I5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: date formatting and images fixes
</commit_message>
<xml_diff>
--- a/SupervisorMobility.API/DataAccess/Templates/Analysis Template.xlsx
+++ b/SupervisorMobility.API/DataAccess/Templates/Analysis Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ituriel\OneDrive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0390C311-95FE-4DA4-885B-F53CDC37E205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6929EFFB-14B0-40C8-8133-B81A9682F52D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29850" yWindow="2025" windowWidth="29835" windowHeight="16605" activeTab="1" xr2:uid="{D0212AFC-6A0E-4C55-A58F-05F4C514B5A6}"/>
+    <workbookView xWindow="4776" yWindow="1920" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{D0212AFC-6A0E-4C55-A58F-05F4C514B5A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Analysis A" sheetId="1" r:id="rId1"/>
@@ -1115,6 +1115,235 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1133,12 +1362,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1146,229 +1369,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1764,163 +1764,163 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:17" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
+      <c r="C3" s="86"/>
+      <c r="D3" s="86"/>
+      <c r="E3" s="86"/>
+      <c r="F3" s="86"/>
+      <c r="G3" s="86"/>
+      <c r="H3" s="86"/>
+      <c r="I3" s="86"/>
+      <c r="J3" s="86"/>
     </row>
     <row r="4" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="56" t="s">
+      <c r="B4" s="87" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="57"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="61"/>
-      <c r="F4" s="61"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="66" t="s">
+      <c r="C4" s="88"/>
+      <c r="D4" s="91"/>
+      <c r="E4" s="92"/>
+      <c r="F4" s="92"/>
+      <c r="G4" s="93"/>
+      <c r="H4" s="97" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="67"/>
-      <c r="J4" s="59"/>
-      <c r="K4" s="89"/>
-      <c r="L4" s="90"/>
-      <c r="M4" s="91"/>
+      <c r="I4" s="98"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="61"/>
+      <c r="L4" s="62"/>
+      <c r="M4" s="63"/>
       <c r="N4" s="12"/>
       <c r="O4" s="12"/>
       <c r="P4" s="11"/>
       <c r="Q4" s="14"/>
     </row>
     <row r="5" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="58"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="63"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="65"/>
-      <c r="H5" s="87" t="s">
+      <c r="B5" s="89"/>
+      <c r="C5" s="90"/>
+      <c r="D5" s="94"/>
+      <c r="E5" s="95"/>
+      <c r="F5" s="95"/>
+      <c r="G5" s="96"/>
+      <c r="H5" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="88"/>
-      <c r="J5" s="86"/>
-      <c r="K5" s="92"/>
-      <c r="L5" s="93"/>
-      <c r="M5" s="94"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="60"/>
+      <c r="K5" s="64"/>
+      <c r="L5" s="65"/>
+      <c r="M5" s="66"/>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
       <c r="P5" s="5"/>
       <c r="Q5" s="14"/>
     </row>
     <row r="6" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="85" t="s">
+      <c r="B6" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="86"/>
-      <c r="D6" s="95"/>
-      <c r="E6" s="96"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="40"/>
       <c r="F6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="G6" s="3"/>
-      <c r="H6" s="101" t="s">
+      <c r="H6" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="102"/>
-      <c r="J6" s="112"/>
-      <c r="K6" s="119"/>
-      <c r="L6" s="119"/>
-      <c r="M6" s="119"/>
-      <c r="N6" s="120"/>
-      <c r="O6" s="121"/>
-      <c r="P6" s="98"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="50"/>
+      <c r="L6" s="50"/>
+      <c r="M6" s="50"/>
+      <c r="N6" s="52"/>
+      <c r="O6" s="53"/>
+      <c r="P6" s="68"/>
     </row>
     <row r="7" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="85" t="s">
+      <c r="B7" s="67" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="86"/>
-      <c r="D7" s="95"/>
-      <c r="E7" s="97"/>
-      <c r="F7" s="97"/>
-      <c r="G7" s="96"/>
-      <c r="H7" s="113"/>
-      <c r="I7" s="114"/>
-      <c r="J7" s="115"/>
-      <c r="K7" s="119"/>
-      <c r="L7" s="119"/>
-      <c r="M7" s="119"/>
-      <c r="N7" s="120"/>
-      <c r="O7" s="122"/>
-      <c r="P7" s="99"/>
+      <c r="C7" s="60"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="40"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="45"/>
+      <c r="J7" s="46"/>
+      <c r="K7" s="50"/>
+      <c r="L7" s="50"/>
+      <c r="M7" s="50"/>
+      <c r="N7" s="52"/>
+      <c r="O7" s="54"/>
+      <c r="P7" s="69"/>
     </row>
     <row r="8" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="85" t="s">
+      <c r="B8" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="86"/>
-      <c r="D8" s="95"/>
-      <c r="E8" s="97"/>
-      <c r="F8" s="97"/>
-      <c r="G8" s="96"/>
-      <c r="H8" s="116"/>
-      <c r="I8" s="117"/>
-      <c r="J8" s="118"/>
-      <c r="K8" s="81"/>
-      <c r="L8" s="81"/>
-      <c r="M8" s="81"/>
-      <c r="N8" s="120"/>
-      <c r="O8" s="123"/>
-      <c r="P8" s="100"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="47"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="49"/>
+      <c r="K8" s="51"/>
+      <c r="L8" s="51"/>
+      <c r="M8" s="51"/>
+      <c r="N8" s="52"/>
+      <c r="O8" s="55"/>
+      <c r="P8" s="70"/>
     </row>
     <row r="9" spans="1:17" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10"/>
-      <c r="B9" s="88" t="s">
+      <c r="B9" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="86"/>
-      <c r="D9" s="95"/>
-      <c r="E9" s="97"/>
-      <c r="F9" s="97"/>
-      <c r="G9" s="96"/>
-      <c r="H9" s="105" t="s">
+      <c r="C9" s="60"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="40"/>
+      <c r="H9" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="101" t="s">
+      <c r="I9" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="J9" s="102"/>
-      <c r="K9" s="80"/>
-      <c r="L9" s="81"/>
-      <c r="M9" s="81"/>
+      <c r="J9" s="42"/>
+      <c r="K9" s="111"/>
+      <c r="L9" s="51"/>
+      <c r="M9" s="51"/>
       <c r="N9" s="6"/>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="14"/>
     </row>
     <row r="10" spans="1:17" ht="46.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="107" t="s">
+      <c r="B10" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="108"/>
-      <c r="D10" s="109"/>
-      <c r="E10" s="110"/>
-      <c r="F10" s="110"/>
-      <c r="G10" s="111"/>
-      <c r="H10" s="106"/>
-      <c r="I10" s="103" t="s">
+      <c r="C10" s="76"/>
+      <c r="D10" s="77"/>
+      <c r="E10" s="78"/>
+      <c r="F10" s="78"/>
+      <c r="G10" s="79"/>
+      <c r="H10" s="74"/>
+      <c r="I10" s="71" t="s">
         <v>10</v>
       </c>
-      <c r="J10" s="104"/>
-      <c r="K10" s="82"/>
-      <c r="L10" s="83"/>
-      <c r="M10" s="84"/>
+      <c r="J10" s="72"/>
+      <c r="K10" s="112"/>
+      <c r="L10" s="113"/>
+      <c r="M10" s="114"/>
       <c r="N10" s="13"/>
       <c r="O10" s="8"/>
       <c r="P10" s="13"/>
@@ -1936,53 +1936,53 @@
       <c r="P11" s="9"/>
     </row>
     <row r="12" spans="1:17" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="68" t="s">
+      <c r="B12" s="99" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="70" t="s">
+      <c r="C12" s="101" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="71"/>
-      <c r="E12" s="74" t="s">
+      <c r="D12" s="102"/>
+      <c r="E12" s="105" t="s">
         <v>14</v>
       </c>
-      <c r="F12" s="70" t="s">
+      <c r="F12" s="101" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="71"/>
-      <c r="H12" s="76" t="s">
+      <c r="G12" s="102"/>
+      <c r="H12" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="76"/>
-      <c r="J12" s="70" t="s">
+      <c r="I12" s="107"/>
+      <c r="J12" s="101" t="s">
         <v>20</v>
       </c>
-      <c r="K12" s="76"/>
-      <c r="L12" s="77"/>
-      <c r="M12" s="44" t="s">
+      <c r="K12" s="107"/>
+      <c r="L12" s="108"/>
+      <c r="M12" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="N12" s="45"/>
-      <c r="O12" s="45"/>
-      <c r="P12" s="45"/>
+      <c r="N12" s="57"/>
+      <c r="O12" s="57"/>
+      <c r="P12" s="57"/>
       <c r="Q12" s="14"/>
     </row>
     <row r="13" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="69"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="73"/>
-      <c r="E13" s="75"/>
-      <c r="F13" s="72"/>
-      <c r="G13" s="73"/>
+      <c r="B13" s="100"/>
+      <c r="C13" s="103"/>
+      <c r="D13" s="104"/>
+      <c r="E13" s="106"/>
+      <c r="F13" s="103"/>
+      <c r="G13" s="104"/>
       <c r="H13" s="17" t="s">
         <v>18</v>
       </c>
       <c r="I13" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="72"/>
-      <c r="K13" s="78"/>
-      <c r="L13" s="79"/>
+      <c r="J13" s="103"/>
+      <c r="K13" s="109"/>
+      <c r="L13" s="110"/>
       <c r="M13" s="16"/>
       <c r="N13" s="9"/>
       <c r="O13" s="9"/>
@@ -1990,29 +1990,29 @@
     </row>
     <row r="14" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="34"/>
-      <c r="C14" s="49"/>
-      <c r="D14" s="52"/>
+      <c r="C14" s="80"/>
+      <c r="D14" s="83"/>
       <c r="E14" s="20"/>
-      <c r="F14" s="53"/>
-      <c r="G14" s="54"/>
+      <c r="F14" s="84"/>
+      <c r="G14" s="85"/>
       <c r="H14" s="18"/>
       <c r="I14" s="19"/>
-      <c r="J14" s="49"/>
-      <c r="K14" s="50"/>
-      <c r="L14" s="51"/>
+      <c r="J14" s="80"/>
+      <c r="K14" s="81"/>
+      <c r="L14" s="82"/>
     </row>
     <row r="15" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="21"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="39"/>
+      <c r="C15" s="115"/>
+      <c r="D15" s="116"/>
       <c r="E15" s="22"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="41"/>
+      <c r="F15" s="117"/>
+      <c r="G15" s="118"/>
       <c r="H15" s="23"/>
       <c r="I15" s="24"/>
-      <c r="J15" s="38"/>
-      <c r="K15" s="42"/>
-      <c r="L15" s="43"/>
+      <c r="J15" s="115"/>
+      <c r="K15" s="119"/>
+      <c r="L15" s="120"/>
     </row>
     <row r="16" spans="1:17" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="27"/>
@@ -2034,35 +2034,53 @@
       <c r="L17" s="26"/>
     </row>
     <row r="18" spans="2:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="44" t="s">
+      <c r="B18" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
+      <c r="C18" s="57"/>
+      <c r="D18" s="57"/>
       <c r="E18" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="F18" s="47" t="s">
+      <c r="F18" s="122" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="45"/>
-      <c r="H18" s="47" t="s">
+      <c r="G18" s="57"/>
+      <c r="H18" s="122" t="s">
         <v>26</v>
       </c>
-      <c r="I18" s="45"/>
-      <c r="J18" s="48"/>
-      <c r="K18" s="45" t="s">
+      <c r="I18" s="57"/>
+      <c r="J18" s="123"/>
+      <c r="K18" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="L18" s="46"/>
+      <c r="L18" s="121"/>
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="H6:J8"/>
-    <mergeCell ref="K6:M8"/>
-    <mergeCell ref="N6:N8"/>
-    <mergeCell ref="O6:O8"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="J15:L15"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="D4:G5"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="F12:G13"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="J12:L13"/>
+    <mergeCell ref="K9:M9"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="B8:C8"/>
     <mergeCell ref="M12:P12"/>
     <mergeCell ref="H5:J5"/>
     <mergeCell ref="K4:M4"/>
@@ -2079,29 +2097,11 @@
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="D10:G10"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="B4:C5"/>
-    <mergeCell ref="D4:G5"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="F12:G13"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J12:L13"/>
-    <mergeCell ref="K9:M9"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="H6:J8"/>
+    <mergeCell ref="K6:M8"/>
+    <mergeCell ref="N6:N8"/>
+    <mergeCell ref="O6:O8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2143,29 +2143,29 @@
     </row>
     <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="68" t="s">
+      <c r="B5" s="99" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="70" t="s">
+      <c r="C5" s="101" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="71"/>
-      <c r="E5" s="74" t="s">
+      <c r="D5" s="102"/>
+      <c r="E5" s="105" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="70" t="s">
+      <c r="F5" s="101" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="71"/>
-      <c r="H5" s="76" t="s">
+      <c r="G5" s="102"/>
+      <c r="H5" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="76"/>
-      <c r="J5" s="70" t="s">
+      <c r="I5" s="107"/>
+      <c r="J5" s="101" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="76"/>
-      <c r="L5" s="77"/>
+      <c r="K5" s="107"/>
+      <c r="L5" s="108"/>
       <c r="M5" s="36" t="s">
         <v>21</v>
       </c>
@@ -2174,21 +2174,21 @@
       <c r="P5" s="35"/>
     </row>
     <row r="6" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="69"/>
-      <c r="C6" s="72"/>
-      <c r="D6" s="73"/>
-      <c r="E6" s="75"/>
-      <c r="F6" s="72"/>
-      <c r="G6" s="73"/>
+      <c r="B6" s="100"/>
+      <c r="C6" s="103"/>
+      <c r="D6" s="104"/>
+      <c r="E6" s="106"/>
+      <c r="F6" s="103"/>
+      <c r="G6" s="104"/>
       <c r="H6" s="17" t="s">
         <v>18</v>
       </c>
       <c r="I6" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="72"/>
-      <c r="K6" s="78"/>
-      <c r="L6" s="79"/>
+      <c r="J6" s="103"/>
+      <c r="K6" s="109"/>
+      <c r="L6" s="110"/>
       <c r="M6" s="16"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.3">
@@ -2237,30 +2237,31 @@
       <c r="L10" s="26"/>
     </row>
     <row r="11" spans="2:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="44" t="s">
+      <c r="B11" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
+      <c r="C11" s="57"/>
+      <c r="D11" s="57"/>
       <c r="E11" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="47" t="s">
+      <c r="F11" s="122" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="45"/>
-      <c r="H11" s="47" t="s">
+      <c r="G11" s="57"/>
+      <c r="H11" s="122" t="s">
         <v>26</v>
       </c>
-      <c r="I11" s="45"/>
-      <c r="J11" s="48"/>
-      <c r="K11" s="45" t="s">
+      <c r="I11" s="57"/>
+      <c r="J11" s="123"/>
+      <c r="K11" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="L11" s="46"/>
+      <c r="L11" s="121"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="F5:G6"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="J5:L6"/>
     <mergeCell ref="B11:D11"/>
@@ -2277,7 +2278,6 @@
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="C5:D6"/>
     <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:G6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: applied sheet generation changes to analysis exportation
</commit_message>
<xml_diff>
--- a/SupervisorMobility.API/DataAccess/Templates/Analysis Template.xlsx
+++ b/SupervisorMobility.API/DataAccess/Templates/Analysis Template.xlsx
@@ -8,14 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ituriel\OneDrive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6929EFFB-14B0-40C8-8133-B81A9682F52D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1028AA4D-CDAB-40B6-8E82-508FBFE8E838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4776" yWindow="1920" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{D0212AFC-6A0E-4C55-A58F-05F4C514B5A6}"/>
+    <workbookView xWindow="32820" yWindow="1350" windowWidth="38700" windowHeight="15285" xr2:uid="{D0212AFC-6A0E-4C55-A58F-05F4C514B5A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Analysis A" sheetId="1" r:id="rId1"/>
-    <sheet name="Analysis B" sheetId="2" r:id="rId2"/>
-    <sheet name="Backup" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <fileRecoveryPr autoRecover="0"/>
@@ -37,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>Nombre del Proceso</t>
   </si>
@@ -125,28 +123,13 @@
   </si>
   <si>
     <t>CANTIDAD</t>
-  </si>
-  <si>
-    <t>Hoja B</t>
-  </si>
-  <si>
-    <t>Supervisor Gral ( Aprobó )</t>
-  </si>
-  <si>
-    <t>Supervisor ( Elaboró )</t>
-  </si>
-  <si>
-    <t>Punto Revisado ( Cambio )</t>
-  </si>
-  <si>
-    <t>No. De Revisión</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,6 +145,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -171,7 +161,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="70">
+  <borders count="69">
     <border>
       <left/>
       <right/>
@@ -999,21 +989,6 @@
     <border>
       <left/>
       <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="medium">
@@ -1028,39 +1003,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1106,22 +1056,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1151,22 +1117,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1184,34 +1150,34 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1232,13 +1198,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1272,22 +1238,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1332,16 +1298,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1370,45 +1336,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1764,297 +1691,297 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:17" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="83" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="86"/>
-      <c r="D3" s="86"/>
-      <c r="E3" s="86"/>
-      <c r="F3" s="86"/>
-      <c r="G3" s="86"/>
-      <c r="H3" s="86"/>
-      <c r="I3" s="86"/>
-      <c r="J3" s="86"/>
+      <c r="C3" s="83"/>
+      <c r="D3" s="83"/>
+      <c r="E3" s="83"/>
+      <c r="F3" s="83"/>
+      <c r="G3" s="83"/>
+      <c r="H3" s="83"/>
+      <c r="I3" s="83"/>
+      <c r="J3" s="83"/>
     </row>
     <row r="4" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="87" t="s">
+      <c r="B4" s="84" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="88"/>
-      <c r="D4" s="91"/>
-      <c r="E4" s="92"/>
-      <c r="F4" s="92"/>
-      <c r="G4" s="93"/>
-      <c r="H4" s="97" t="s">
+      <c r="C4" s="85"/>
+      <c r="D4" s="88"/>
+      <c r="E4" s="89"/>
+      <c r="F4" s="89"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="98"/>
-      <c r="J4" s="90"/>
-      <c r="K4" s="61"/>
-      <c r="L4" s="62"/>
-      <c r="M4" s="63"/>
-      <c r="N4" s="12"/>
-      <c r="O4" s="12"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="14"/>
+      <c r="I4" s="95"/>
+      <c r="J4" s="87"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="59"/>
+      <c r="M4" s="60"/>
+      <c r="N4" s="33"/>
+      <c r="O4" s="33"/>
+      <c r="P4" s="27"/>
+      <c r="Q4" s="5"/>
     </row>
     <row r="5" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="89"/>
-      <c r="C5" s="90"/>
-      <c r="D5" s="94"/>
-      <c r="E5" s="95"/>
-      <c r="F5" s="95"/>
-      <c r="G5" s="96"/>
-      <c r="H5" s="58" t="s">
+      <c r="B5" s="86"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="91"/>
+      <c r="E5" s="92"/>
+      <c r="F5" s="92"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="59"/>
-      <c r="J5" s="60"/>
-      <c r="K5" s="64"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="66"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="7"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="14"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="57"/>
+      <c r="K5" s="61"/>
+      <c r="L5" s="62"/>
+      <c r="M5" s="63"/>
+      <c r="N5" s="32"/>
+      <c r="O5" s="32"/>
+      <c r="P5" s="28"/>
+      <c r="Q5" s="5"/>
     </row>
     <row r="6" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="67" t="s">
+      <c r="B6" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="60"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="40"/>
+      <c r="C6" s="57"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="37"/>
       <c r="F6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="41" t="s">
+      <c r="G6" s="26"/>
+      <c r="H6" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="42"/>
-      <c r="J6" s="43"/>
-      <c r="K6" s="50"/>
-      <c r="L6" s="50"/>
-      <c r="M6" s="50"/>
-      <c r="N6" s="52"/>
-      <c r="O6" s="53"/>
-      <c r="P6" s="68"/>
+      <c r="I6" s="39"/>
+      <c r="J6" s="40"/>
+      <c r="K6" s="47"/>
+      <c r="L6" s="47"/>
+      <c r="M6" s="47"/>
+      <c r="N6" s="49"/>
+      <c r="O6" s="50"/>
+      <c r="P6" s="65"/>
     </row>
     <row r="7" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="67" t="s">
+      <c r="B7" s="64" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="60"/>
-      <c r="D7" s="38"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
-      <c r="G7" s="40"/>
-      <c r="H7" s="44"/>
-      <c r="I7" s="45"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="50"/>
-      <c r="L7" s="50"/>
-      <c r="M7" s="50"/>
-      <c r="N7" s="52"/>
-      <c r="O7" s="54"/>
-      <c r="P7" s="69"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="41"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="43"/>
+      <c r="K7" s="47"/>
+      <c r="L7" s="47"/>
+      <c r="M7" s="47"/>
+      <c r="N7" s="49"/>
+      <c r="O7" s="51"/>
+      <c r="P7" s="66"/>
     </row>
     <row r="8" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="67" t="s">
+      <c r="B8" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="60"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="47"/>
-      <c r="I8" s="48"/>
-      <c r="J8" s="49"/>
-      <c r="K8" s="51"/>
-      <c r="L8" s="51"/>
-      <c r="M8" s="51"/>
-      <c r="N8" s="52"/>
-      <c r="O8" s="55"/>
-      <c r="P8" s="70"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="45"/>
+      <c r="J8" s="46"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="48"/>
+      <c r="M8" s="48"/>
+      <c r="N8" s="49"/>
+      <c r="O8" s="52"/>
+      <c r="P8" s="67"/>
     </row>
     <row r="9" spans="1:17" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10"/>
-      <c r="B9" s="59" t="s">
+      <c r="A9" s="4"/>
+      <c r="B9" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="60"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="40"/>
-      <c r="H9" s="73" t="s">
+      <c r="C9" s="57"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="70" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="41" t="s">
+      <c r="I9" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="J9" s="42"/>
-      <c r="K9" s="111"/>
-      <c r="L9" s="51"/>
-      <c r="M9" s="51"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="4"/>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="14"/>
+      <c r="J9" s="39"/>
+      <c r="K9" s="108"/>
+      <c r="L9" s="48"/>
+      <c r="M9" s="48"/>
+      <c r="N9" s="30"/>
+      <c r="O9" s="31"/>
+      <c r="P9" s="31"/>
+      <c r="Q9" s="5"/>
     </row>
     <row r="10" spans="1:17" ht="46.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="75" t="s">
+      <c r="B10" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="76"/>
-      <c r="D10" s="77"/>
-      <c r="E10" s="78"/>
-      <c r="F10" s="78"/>
-      <c r="G10" s="79"/>
-      <c r="H10" s="74"/>
-      <c r="I10" s="71" t="s">
+      <c r="C10" s="73"/>
+      <c r="D10" s="74"/>
+      <c r="E10" s="75"/>
+      <c r="F10" s="75"/>
+      <c r="G10" s="76"/>
+      <c r="H10" s="71"/>
+      <c r="I10" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="J10" s="72"/>
-      <c r="K10" s="112"/>
-      <c r="L10" s="113"/>
-      <c r="M10" s="114"/>
-      <c r="N10" s="13"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="13"/>
-      <c r="Q10" s="14"/>
+      <c r="J10" s="69"/>
+      <c r="K10" s="109"/>
+      <c r="L10" s="110"/>
+      <c r="M10" s="111"/>
+      <c r="N10" s="29"/>
+      <c r="O10" s="34"/>
+      <c r="P10" s="29"/>
+      <c r="Q10" s="5"/>
     </row>
     <row r="11" spans="1:17" ht="9.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="E11" s="15"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="E11" s="6"/>
       <c r="H11" s="1"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
     </row>
     <row r="12" spans="1:17" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="99" t="s">
+      <c r="B12" s="96" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="101" t="s">
+      <c r="C12" s="98" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="102"/>
-      <c r="E12" s="105" t="s">
+      <c r="D12" s="99"/>
+      <c r="E12" s="102" t="s">
         <v>14</v>
       </c>
-      <c r="F12" s="101" t="s">
+      <c r="F12" s="98" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="102"/>
-      <c r="H12" s="107" t="s">
+      <c r="G12" s="99"/>
+      <c r="H12" s="104" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="107"/>
-      <c r="J12" s="101" t="s">
+      <c r="I12" s="104"/>
+      <c r="J12" s="98" t="s">
         <v>20</v>
       </c>
-      <c r="K12" s="107"/>
-      <c r="L12" s="108"/>
-      <c r="M12" s="56" t="s">
+      <c r="K12" s="104"/>
+      <c r="L12" s="105"/>
+      <c r="M12" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="N12" s="57"/>
-      <c r="O12" s="57"/>
-      <c r="P12" s="57"/>
-      <c r="Q12" s="14"/>
+      <c r="N12" s="54"/>
+      <c r="O12" s="54"/>
+      <c r="P12" s="54"/>
+      <c r="Q12" s="5"/>
     </row>
     <row r="13" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="100"/>
-      <c r="C13" s="103"/>
-      <c r="D13" s="104"/>
-      <c r="E13" s="106"/>
-      <c r="F13" s="103"/>
-      <c r="G13" s="104"/>
-      <c r="H13" s="17" t="s">
+      <c r="B13" s="97"/>
+      <c r="C13" s="100"/>
+      <c r="D13" s="101"/>
+      <c r="E13" s="103"/>
+      <c r="F13" s="100"/>
+      <c r="G13" s="101"/>
+      <c r="H13" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="17" t="s">
+      <c r="I13" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="103"/>
-      <c r="K13" s="109"/>
-      <c r="L13" s="110"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="9"/>
+      <c r="J13" s="100"/>
+      <c r="K13" s="106"/>
+      <c r="L13" s="107"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="3"/>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
     </row>
     <row r="14" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="34"/>
-      <c r="C14" s="80"/>
-      <c r="D14" s="83"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="84"/>
-      <c r="G14" s="85"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="19"/>
-      <c r="J14" s="80"/>
-      <c r="K14" s="81"/>
-      <c r="L14" s="82"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="80"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="81"/>
+      <c r="G14" s="82"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="77"/>
+      <c r="K14" s="78"/>
+      <c r="L14" s="79"/>
     </row>
     <row r="15" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="21"/>
-      <c r="C15" s="115"/>
-      <c r="D15" s="116"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="117"/>
-      <c r="G15" s="118"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="115"/>
-      <c r="K15" s="119"/>
-      <c r="L15" s="120"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="113"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="114"/>
+      <c r="G15" s="115"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="112"/>
+      <c r="K15" s="116"/>
+      <c r="L15" s="117"/>
     </row>
     <row r="16" spans="1:17" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="27"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="29" t="s">
+      <c r="B16" s="18"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="H16" s="30"/>
-      <c r="I16" s="32"/>
-      <c r="J16" s="30"/>
-      <c r="K16" s="28"/>
-      <c r="L16" s="31"/>
+      <c r="H16" s="21"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="21"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="22"/>
     </row>
     <row r="17" spans="2:12" ht="7.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="25"/>
-      <c r="L17" s="26"/>
+      <c r="B17" s="16"/>
+      <c r="L17" s="17"/>
     </row>
     <row r="18" spans="2:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="56" t="s">
+      <c r="B18" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="57"/>
-      <c r="D18" s="57"/>
-      <c r="E18" s="33" t="s">
+      <c r="C18" s="54"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="F18" s="122" t="s">
+      <c r="F18" s="119" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="57"/>
-      <c r="H18" s="122" t="s">
+      <c r="G18" s="54"/>
+      <c r="H18" s="119" t="s">
         <v>26</v>
       </c>
-      <c r="I18" s="57"/>
-      <c r="J18" s="123"/>
-      <c r="K18" s="57" t="s">
+      <c r="I18" s="54"/>
+      <c r="J18" s="120"/>
+      <c r="K18" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="L18" s="121"/>
+      <c r="L18" s="118"/>
     </row>
   </sheetData>
   <mergeCells count="44">
@@ -2106,212 +2033,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C7884FB-B74C-4B2A-8E22-E86C0746225B}">
-  <dimension ref="B3:P11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="5.77734375" customWidth="1"/>
-    <col min="3" max="3" width="30.77734375" customWidth="1"/>
-    <col min="4" max="4" width="20.77734375" customWidth="1"/>
-    <col min="5" max="5" width="10.77734375" customWidth="1"/>
-    <col min="6" max="6" width="30.77734375" customWidth="1"/>
-    <col min="7" max="7" width="20.77734375" customWidth="1"/>
-    <col min="8" max="8" width="7.77734375" customWidth="1"/>
-    <col min="9" max="9" width="6.77734375" customWidth="1"/>
-    <col min="10" max="10" width="15.77734375" customWidth="1"/>
-    <col min="11" max="11" width="8.77734375" customWidth="1"/>
-    <col min="12" max="12" width="18.6640625" customWidth="1"/>
-    <col min="13" max="13" width="96.77734375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="2:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B3" s="124" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="124"/>
-      <c r="D3" s="124"/>
-      <c r="E3" s="124"/>
-      <c r="F3" s="124"/>
-      <c r="G3" s="124"/>
-      <c r="H3" s="124"/>
-      <c r="I3" s="124"/>
-      <c r="J3" s="124"/>
-    </row>
-    <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="2:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="99" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="101" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="102"/>
-      <c r="E5" s="105" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="101" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="102"/>
-      <c r="H5" s="107" t="s">
-        <v>17</v>
-      </c>
-      <c r="I5" s="107"/>
-      <c r="J5" s="101" t="s">
-        <v>20</v>
-      </c>
-      <c r="K5" s="107"/>
-      <c r="L5" s="108"/>
-      <c r="M5" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="N5" s="35"/>
-      <c r="O5" s="35"/>
-      <c r="P5" s="35"/>
-    </row>
-    <row r="6" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="100"/>
-      <c r="C6" s="103"/>
-      <c r="D6" s="104"/>
-      <c r="E6" s="106"/>
-      <c r="F6" s="103"/>
-      <c r="G6" s="104"/>
-      <c r="H6" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="I6" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="J6" s="103"/>
-      <c r="K6" s="109"/>
-      <c r="L6" s="110"/>
-      <c r="M6" s="16"/>
-    </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B7" s="34"/>
-      <c r="C7" s="125"/>
-      <c r="D7" s="126"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="127"/>
-      <c r="G7" s="128"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="125"/>
-      <c r="K7" s="129"/>
-      <c r="L7" s="130"/>
-    </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B8" s="21"/>
-      <c r="C8" s="131"/>
-      <c r="D8" s="132"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="133"/>
-      <c r="G8" s="134"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="24"/>
-      <c r="J8" s="131"/>
-      <c r="K8" s="135"/>
-      <c r="L8" s="136"/>
-    </row>
-    <row r="9" spans="2:16" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="27"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="H9" s="30"/>
-      <c r="I9" s="32"/>
-      <c r="J9" s="30"/>
-      <c r="K9" s="28"/>
-      <c r="L9" s="31"/>
-    </row>
-    <row r="10" spans="2:16" ht="7.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="25"/>
-      <c r="L10" s="26"/>
-    </row>
-    <row r="11" spans="2:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="56" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="57"/>
-      <c r="D11" s="57"/>
-      <c r="E11" s="33" t="s">
-        <v>24</v>
-      </c>
-      <c r="F11" s="122" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11" s="57"/>
-      <c r="H11" s="122" t="s">
-        <v>26</v>
-      </c>
-      <c r="I11" s="57"/>
-      <c r="J11" s="123"/>
-      <c r="K11" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="L11" s="121"/>
-    </row>
-  </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="F5:G6"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:L6"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="J8:L8"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:D6"/>
-    <mergeCell ref="E5:E6"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BF89785-B436-4CCD-AC9F-CFA0D9BC19AA}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="2" width="55.77734375" customWidth="1"/>
-    <col min="3" max="3" width="162.77734375" customWidth="1"/>
-    <col min="4" max="5" width="55.77734375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="37" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="37" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2" s="37" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" s="37" t="s">
-        <v>30</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: removed comments from exportation controller
</commit_message>
<xml_diff>
--- a/SupervisorMobility.API/DataAccess/Templates/Analysis Template.xlsx
+++ b/SupervisorMobility.API/DataAccess/Templates/Analysis Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ituriel\OneDrive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1028AA4D-CDAB-40B6-8E82-508FBFE8E838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B795CC17-9CEF-4A66-925B-36488DFCA7E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32820" yWindow="1350" windowWidth="38700" windowHeight="15285" xr2:uid="{D0212AFC-6A0E-4C55-A58F-05F4C514B5A6}"/>
+    <workbookView xWindow="29760" yWindow="960" windowWidth="38700" windowHeight="15285" xr2:uid="{D0212AFC-6A0E-4C55-A58F-05F4C514B5A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Analysis A" sheetId="1" r:id="rId1"/>
@@ -161,7 +161,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="69">
+  <borders count="72">
     <border>
       <left/>
       <right/>
@@ -992,6 +992,51 @@
         <color indexed="64"/>
       </right>
       <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
@@ -1003,7 +1048,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1011,7 +1056,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1059,12 +1103,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1081,6 +1119,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1141,6 +1189,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1327,9 +1378,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1671,7 +1719,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{046F2C6B-7280-4C6F-BF6B-1D857D75FA49}">
-  <dimension ref="A3:Q18"/>
+  <dimension ref="A3:P18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="0.88671875" customWidth="1"/>
@@ -1690,298 +1738,293 @@
     <col min="14" max="16" width="30.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:17" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="83" t="s">
+    <row r="3" spans="1:16" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="85" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="83"/>
-      <c r="I3" s="83"/>
-      <c r="J3" s="83"/>
+      <c r="C3" s="85"/>
+      <c r="D3" s="85"/>
+      <c r="E3" s="85"/>
+      <c r="F3" s="85"/>
+      <c r="G3" s="85"/>
+      <c r="H3" s="85"/>
+      <c r="I3" s="85"/>
+      <c r="J3" s="85"/>
     </row>
-    <row r="4" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="84" t="s">
+    <row r="4" spans="1:16" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="85"/>
-      <c r="D4" s="88"/>
-      <c r="E4" s="89"/>
-      <c r="F4" s="89"/>
-      <c r="G4" s="90"/>
-      <c r="H4" s="94" t="s">
+      <c r="C4" s="87"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="91"/>
+      <c r="F4" s="91"/>
+      <c r="G4" s="92"/>
+      <c r="H4" s="96" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="95"/>
-      <c r="J4" s="87"/>
-      <c r="K4" s="58"/>
-      <c r="L4" s="59"/>
-      <c r="M4" s="60"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="33"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="5"/>
+      <c r="I4" s="97"/>
+      <c r="J4" s="89"/>
+      <c r="K4" s="60"/>
+      <c r="L4" s="61"/>
+      <c r="M4" s="62"/>
+      <c r="N4" s="30"/>
+      <c r="O4" s="30"/>
+      <c r="P4" s="32"/>
     </row>
-    <row r="5" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="86"/>
-      <c r="C5" s="87"/>
-      <c r="D5" s="91"/>
-      <c r="E5" s="92"/>
-      <c r="F5" s="92"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="55" t="s">
+    <row r="5" spans="1:16" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="88"/>
+      <c r="C5" s="89"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="94"/>
+      <c r="F5" s="94"/>
+      <c r="G5" s="95"/>
+      <c r="H5" s="57" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="56"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="61"/>
-      <c r="L5" s="62"/>
-      <c r="M5" s="63"/>
-      <c r="N5" s="32"/>
-      <c r="O5" s="32"/>
-      <c r="P5" s="28"/>
-      <c r="Q5" s="5"/>
+      <c r="I5" s="58"/>
+      <c r="J5" s="59"/>
+      <c r="K5" s="63"/>
+      <c r="L5" s="64"/>
+      <c r="M5" s="65"/>
+      <c r="N5" s="29"/>
+      <c r="O5" s="29"/>
+      <c r="P5" s="33"/>
     </row>
-    <row r="6" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="64" t="s">
+    <row r="6" spans="1:16" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="57"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="37"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="38"/>
       <c r="F6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="G6" s="26"/>
-      <c r="H6" s="38" t="s">
+      <c r="G6" s="25"/>
+      <c r="H6" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="39"/>
-      <c r="J6" s="40"/>
-      <c r="K6" s="47"/>
-      <c r="L6" s="47"/>
-      <c r="M6" s="47"/>
-      <c r="N6" s="49"/>
-      <c r="O6" s="50"/>
-      <c r="P6" s="65"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="48"/>
+      <c r="L6" s="48"/>
+      <c r="M6" s="48"/>
+      <c r="N6" s="50"/>
+      <c r="O6" s="51"/>
+      <c r="P6" s="67"/>
     </row>
-    <row r="7" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="64" t="s">
+    <row r="7" spans="1:16" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="57"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="41"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="43"/>
-      <c r="K7" s="47"/>
-      <c r="L7" s="47"/>
-      <c r="M7" s="47"/>
-      <c r="N7" s="49"/>
-      <c r="O7" s="51"/>
-      <c r="P7" s="66"/>
+      <c r="C7" s="59"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="38"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="48"/>
+      <c r="L7" s="48"/>
+      <c r="M7" s="48"/>
+      <c r="N7" s="50"/>
+      <c r="O7" s="52"/>
+      <c r="P7" s="68"/>
     </row>
-    <row r="8" spans="1:17" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="64" t="s">
+    <row r="8" spans="1:16" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="66" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="57"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="44"/>
-      <c r="I8" s="45"/>
-      <c r="J8" s="46"/>
-      <c r="K8" s="48"/>
-      <c r="L8" s="48"/>
-      <c r="M8" s="48"/>
-      <c r="N8" s="49"/>
-      <c r="O8" s="52"/>
-      <c r="P8" s="67"/>
+      <c r="C8" s="59"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="45"/>
+      <c r="I8" s="46"/>
+      <c r="J8" s="47"/>
+      <c r="K8" s="49"/>
+      <c r="L8" s="49"/>
+      <c r="M8" s="49"/>
+      <c r="N8" s="50"/>
+      <c r="O8" s="53"/>
+      <c r="P8" s="69"/>
     </row>
-    <row r="9" spans="1:17" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="B9" s="56" t="s">
+      <c r="B9" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="57"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="70" t="s">
+      <c r="C9" s="59"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="38"/>
+      <c r="H9" s="72" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="38" t="s">
+      <c r="I9" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="J9" s="39"/>
-      <c r="K9" s="108"/>
-      <c r="L9" s="48"/>
-      <c r="M9" s="48"/>
-      <c r="N9" s="30"/>
-      <c r="O9" s="31"/>
-      <c r="P9" s="31"/>
-      <c r="Q9" s="5"/>
+      <c r="J9" s="40"/>
+      <c r="K9" s="110"/>
+      <c r="L9" s="49"/>
+      <c r="M9" s="49"/>
+      <c r="N9" s="27"/>
+      <c r="O9" s="28"/>
+      <c r="P9" s="33"/>
     </row>
-    <row r="10" spans="1:17" ht="46.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="72" t="s">
+    <row r="10" spans="1:16" ht="46.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="73"/>
-      <c r="D10" s="74"/>
-      <c r="E10" s="75"/>
-      <c r="F10" s="75"/>
-      <c r="G10" s="76"/>
-      <c r="H10" s="71"/>
-      <c r="I10" s="68" t="s">
+      <c r="C10" s="75"/>
+      <c r="D10" s="76"/>
+      <c r="E10" s="77"/>
+      <c r="F10" s="77"/>
+      <c r="G10" s="78"/>
+      <c r="H10" s="73"/>
+      <c r="I10" s="70" t="s">
         <v>10</v>
       </c>
-      <c r="J10" s="69"/>
-      <c r="K10" s="109"/>
-      <c r="L10" s="110"/>
-      <c r="M10" s="111"/>
-      <c r="N10" s="29"/>
-      <c r="O10" s="34"/>
-      <c r="P10" s="29"/>
-      <c r="Q10" s="5"/>
+      <c r="J10" s="71"/>
+      <c r="K10" s="111"/>
+      <c r="L10" s="112"/>
+      <c r="M10" s="113"/>
+      <c r="N10" s="26"/>
+      <c r="O10" s="31"/>
+      <c r="P10" s="34"/>
     </row>
-    <row r="11" spans="1:17" ht="9.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" ht="9.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
-      <c r="E11" s="6"/>
+      <c r="E11" s="5"/>
       <c r="H11" s="1"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
-      <c r="P11" s="3"/>
+      <c r="P11" s="35"/>
     </row>
-    <row r="12" spans="1:17" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="96" t="s">
+    <row r="12" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="98" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="98" t="s">
+      <c r="C12" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="99"/>
-      <c r="E12" s="102" t="s">
+      <c r="D12" s="101"/>
+      <c r="E12" s="104" t="s">
         <v>14</v>
       </c>
-      <c r="F12" s="98" t="s">
+      <c r="F12" s="100" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="99"/>
-      <c r="H12" s="104" t="s">
+      <c r="G12" s="101"/>
+      <c r="H12" s="106" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="104"/>
-      <c r="J12" s="98" t="s">
+      <c r="I12" s="106"/>
+      <c r="J12" s="100" t="s">
         <v>20</v>
       </c>
-      <c r="K12" s="104"/>
-      <c r="L12" s="105"/>
-      <c r="M12" s="53" t="s">
+      <c r="K12" s="106"/>
+      <c r="L12" s="107"/>
+      <c r="M12" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="N12" s="54"/>
-      <c r="O12" s="54"/>
-      <c r="P12" s="54"/>
-      <c r="Q12" s="5"/>
+      <c r="N12" s="55"/>
+      <c r="O12" s="55"/>
+      <c r="P12" s="56"/>
     </row>
-    <row r="13" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="97"/>
-      <c r="C13" s="100"/>
-      <c r="D13" s="101"/>
-      <c r="E13" s="103"/>
-      <c r="F13" s="100"/>
-      <c r="G13" s="101"/>
-      <c r="H13" s="8" t="s">
+    <row r="13" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="99"/>
+      <c r="C13" s="102"/>
+      <c r="D13" s="103"/>
+      <c r="E13" s="105"/>
+      <c r="F13" s="102"/>
+      <c r="G13" s="103"/>
+      <c r="H13" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="8" t="s">
+      <c r="I13" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="100"/>
-      <c r="K13" s="106"/>
-      <c r="L13" s="107"/>
-      <c r="M13" s="7"/>
+      <c r="J13" s="102"/>
+      <c r="K13" s="108"/>
+      <c r="L13" s="109"/>
+      <c r="M13" s="6"/>
       <c r="N13" s="3"/>
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
     </row>
-    <row r="14" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="25"/>
-      <c r="C14" s="77"/>
-      <c r="D14" s="80"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="81"/>
-      <c r="G14" s="82"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="77"/>
-      <c r="K14" s="78"/>
-      <c r="L14" s="79"/>
+    <row r="14" spans="1:16" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="24"/>
+      <c r="C14" s="79"/>
+      <c r="D14" s="82"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="83"/>
+      <c r="G14" s="84"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="79"/>
+      <c r="K14" s="80"/>
+      <c r="L14" s="81"/>
     </row>
-    <row r="15" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="12"/>
-      <c r="C15" s="112"/>
-      <c r="D15" s="113"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="114"/>
-      <c r="G15" s="115"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="112"/>
-      <c r="K15" s="116"/>
-      <c r="L15" s="117"/>
+    <row r="15" spans="1:16" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="11"/>
+      <c r="C15" s="114"/>
+      <c r="D15" s="115"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="116"/>
+      <c r="G15" s="117"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="114"/>
+      <c r="K15" s="118"/>
+      <c r="L15" s="119"/>
     </row>
-    <row r="16" spans="1:17" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="18"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="20" t="s">
+    <row r="16" spans="1:16" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="17"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="H16" s="21"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="21"/>
-      <c r="K16" s="19"/>
-      <c r="L16" s="22"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="22"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="21"/>
     </row>
     <row r="17" spans="2:12" ht="7.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="16"/>
-      <c r="L17" s="17"/>
+      <c r="B17" s="15"/>
+      <c r="L17" s="16"/>
     </row>
     <row r="18" spans="2:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="53" t="s">
+      <c r="B18" s="54" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="54"/>
-      <c r="D18" s="54"/>
-      <c r="E18" s="24" t="s">
+      <c r="C18" s="55"/>
+      <c r="D18" s="55"/>
+      <c r="E18" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="F18" s="119" t="s">
+      <c r="F18" s="120" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="54"/>
-      <c r="H18" s="119" t="s">
+      <c r="G18" s="55"/>
+      <c r="H18" s="120" t="s">
         <v>26</v>
       </c>
-      <c r="I18" s="54"/>
-      <c r="J18" s="120"/>
-      <c r="K18" s="54" t="s">
+      <c r="I18" s="55"/>
+      <c r="J18" s="121"/>
+      <c r="K18" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="L18" s="118"/>
+      <c r="L18" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="44">

</xml_diff>